<commit_message>
rutificador implementado y correcion excel
</commit_message>
<xml_diff>
--- a/src/main/resources/static/ayy.xlsx
+++ b/src/main/resources/static/ayy.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="12">
   <si>
     <t xml:space="preserve">N.º</t>
   </si>
@@ -31,10 +31,31 @@
     <t xml:space="preserve">correo</t>
   </si>
   <si>
+    <t xml:space="preserve">rut</t>
+  </si>
+  <si>
+    <t xml:space="preserve">rutificador</t>
+  </si>
+  <si>
     <t xml:space="preserve">javier ulloa fierro</t>
   </si>
   <si>
     <t xml:space="preserve">javierulloafierro@gmail.com</t>
+  </si>
+  <si>
+    <t xml:space="preserve">si</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pedro test</t>
+  </si>
+  <si>
+    <t xml:space="preserve">16.163.631-2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">juan test</t>
+  </si>
+  <si>
+    <t xml:space="preserve">no</t>
   </si>
 </sst>
 </file>
@@ -45,7 +66,7 @@
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="[$€-410]\ #,##0.00;[RED]\-[$€-410]\ #,##0.00"/>
   </numFmts>
-  <fonts count="6">
+  <fonts count="7">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -71,6 +92,12 @@
       <u val="single"/>
       <sz val="10"/>
       <name val="Lohit Hindi"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="arial"/>
       <family val="2"/>
       <charset val="1"/>
     </font>
@@ -127,12 +154,20 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -260,34 +295,81 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:C2"/>
+  <dimension ref="A1:E4"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="23.97"/>
+  </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="0" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="0" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="0" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
+      </c>
+      <c r="D1" s="0" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>4</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="0" t="n">
+      <c r="A2" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="0" t="s">
+      <c r="B2" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="D2" s="0" t="n">
+        <v>212650455</v>
+      </c>
+      <c r="E2" s="0" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E3" s="0" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="0" t="n">
         <v>3</v>
       </c>
-      <c r="C2" s="1" t="s">
-        <v>4</v>
+      <c r="B4" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E4" s="0" t="s">
+        <v>11</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="C2" r:id="rId1" display="javierulloafierro@gmail.com"/>
+    <hyperlink ref="C3" r:id="rId2" display="javierulloafierro@gmail.com"/>
   </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.025" bottom="1.025" header="0.7875" footer="0.7875"/>

</xml_diff>